<commit_message>
Stage 8 review fixes: A-021
</commit_message>
<xml_diff>
--- a/output/archive/Archive/Users/omerriman_old_laptop/Commercial/2021/VD_price_grid_18Nov21_revC.xlsx
+++ b/output/archive/Archive/Users/omerriman_old_laptop/Commercial/2021/VD_price_grid_18Nov21_revC.xlsx
@@ -562,7 +562,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>per impurity</t>
+          <t>Scope dependent</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Price not agreed; priced per programme for now</t>
+          <t>No list price; quote separately after programme review</t>
         </is>
       </c>
     </row>
@@ -606,142 +606,121 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Approval note</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Discount basis</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>Requested</t>
+          <t>Approval record</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>Approved by</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>Outcome</t>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>08 Mar 2021</t>
+          <t>Historical framework enquiry</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Client on the 2020 framework</t>
+          <t>Analogue preparation</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Analogue preparation</t>
+          <t>Exception to list bands</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Extra 3% on the 30 compound band</t>
+          <t>Refer to commercial approval notes</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Eleanor Vellacombe</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Approved for that programme only</t>
+          <t>Check before reuse</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>27 Jul 2021</t>
+          <t>Historical scout-fee enquiry</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>New enquiry</t>
+          <t>Route scout and delivery</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Route scout and delivery</t>
+          <t>No list discount</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Route fee waived for the scout step</t>
+          <t>Refer to commercial approval notes</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Ruth Calderwood</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Declined. Scout fee stands.</t>
+          <t>Check before reuse</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>19 Oct 2021</t>
+          <t>Historical volume-band enquiry</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Existing client</t>
+          <t>Analogue preparation</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Analogue preparation</t>
+          <t>Exception to list bands</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>10% band at 40 compounds</t>
+          <t>Refer to commercial approval notes</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Eleanor Vellacombe</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Approved, subject to a signed programme</t>
+          <t>Check before reuse</t>
         </is>
       </c>
     </row>
@@ -752,7 +731,6 @@
       <c r="C6" s="3" t="inlineStr"/>
       <c r="D6" s="3" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -783,14 +761,14 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>The 10% band starts above 80 compounds. Quotes between 30 and 80 compounds take the 5% band.</t>
+          <t>The 5% band applies above 30 compounds up to and including 80; the 10% band applies above 80. No list discount applies at 30 compounds.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Route scout fees are not discounted. Ruth has asked us to keep it that way.</t>
+          <t>Route scout and delivery has no list discount. Check the approval record before reusing a historical exception.</t>
         </is>
       </c>
     </row>

</xml_diff>